<commit_message>
update sector path wb
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_morocco_transformation_cw.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_morocco_transformation_cw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_morocco/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6AE2884-094E-1E44-9BB0-3F11BEB7D84F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D806F3-EF87-1C4E-891D-063E089CCC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-43800" yWindow="600" windowWidth="36440" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-51200" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -2114,7 +2114,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:R70"/>
@@ -2183,7 +2183,7 @@
       <c r="Q1" s="11"/>
       <c r="R1" s="11"/>
     </row>
-    <row r="2" spans="1:18" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" s="4" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>212</v>
       </c>
@@ -2222,7 +2222,7 @@
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
     </row>
-    <row r="3" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>212</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>1.8</v>
       </c>
       <c r="N3" s="17">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="O3" s="10"/>
       <c r="P3" s="10">
@@ -2265,7 +2265,7 @@
       <c r="Q3" s="11"/>
       <c r="R3" s="11"/>
     </row>
-    <row r="4" spans="1:18" s="4" customFormat="1" ht="86" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" s="4" customFormat="1" ht="86" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>212</v>
       </c>
@@ -2297,9 +2297,7 @@
       <c r="M4" s="17">
         <v>1.5</v>
       </c>
-      <c r="N4" s="17">
-        <v>1.5</v>
-      </c>
+      <c r="N4" s="17"/>
       <c r="O4" s="10"/>
       <c r="P4" s="10">
         <f t="shared" si="0"/>
@@ -2310,7 +2308,7 @@
       </c>
       <c r="R4" s="11"/>
     </row>
-    <row r="5" spans="1:18" s="4" customFormat="1" ht="153" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" s="4" customFormat="1" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>212</v>
       </c>
@@ -2342,9 +2340,7 @@
       <c r="M5" s="17">
         <v>1</v>
       </c>
-      <c r="N5" s="17">
-        <v>1</v>
-      </c>
+      <c r="N5" s="17"/>
       <c r="O5" s="10"/>
       <c r="P5" s="10" t="e">
         <f t="shared" si="0"/>
@@ -2353,7 +2349,7 @@
       <c r="Q5" s="11"/>
       <c r="R5" s="11"/>
     </row>
-    <row r="6" spans="1:18" s="4" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" s="4" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>212</v>
       </c>
@@ -2389,9 +2385,7 @@
       <c r="M6" s="17">
         <v>4.5</v>
       </c>
-      <c r="N6" s="17">
-        <v>5</v>
-      </c>
+      <c r="N6" s="17"/>
       <c r="O6" s="10"/>
       <c r="P6" s="10">
         <f>0.6*M6</f>
@@ -2399,11 +2393,11 @@
       </c>
       <c r="Q6" s="10">
         <f>K6*N6</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
         <v>226</v>
       </c>
@@ -2442,7 +2436,7 @@
       <c r="Q7" s="11"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" s="4" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" s="4" customFormat="1" ht="55" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>226</v>
       </c>
@@ -2492,7 +2486,7 @@
       </c>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>226</v>
       </c>
@@ -2539,7 +2533,7 @@
       <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
     </row>
-    <row r="10" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>226</v>
       </c>
@@ -2586,7 +2580,7 @@
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
     </row>
-    <row r="11" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
         <v>226</v>
       </c>
@@ -2630,7 +2624,7 @@
       </c>
       <c r="R11" s="11"/>
     </row>
-    <row r="12" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>226</v>
       </c>
@@ -2676,7 +2670,7 @@
       </c>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
         <v>226</v>
       </c>
@@ -2721,7 +2715,7 @@
       </c>
       <c r="R13" s="11"/>
     </row>
-    <row r="14" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>226</v>
       </c>
@@ -2771,7 +2765,7 @@
       </c>
       <c r="R14" s="11"/>
     </row>
-    <row r="15" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
         <v>226</v>
       </c>
@@ -2821,7 +2815,7 @@
       </c>
       <c r="R15" s="11"/>
     </row>
-    <row r="16" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
         <v>226</v>
       </c>
@@ -2861,7 +2855,7 @@
       <c r="Q16" s="11"/>
       <c r="R16" s="11"/>
     </row>
-    <row r="17" spans="1:18" s="58" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" s="58" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="s">
         <v>51</v>
       </c>
@@ -2898,7 +2892,7 @@
         <v>1.5</v>
       </c>
       <c r="N17" s="72">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="O17" s="10"/>
       <c r="P17" s="10">
@@ -2907,11 +2901,11 @@
       </c>
       <c r="Q17" s="10">
         <f t="shared" ref="Q17:Q22" si="3">K17*N17</f>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="R17" s="57"/>
     </row>
-    <row r="18" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
         <v>51</v>
       </c>
@@ -2947,8 +2941,8 @@
       <c r="M18" s="71">
         <v>2</v>
       </c>
-      <c r="N18" s="71">
-        <v>2</v>
+      <c r="N18" s="72">
+        <v>1</v>
       </c>
       <c r="O18" s="10"/>
       <c r="P18" s="10">
@@ -2957,11 +2951,11 @@
       </c>
       <c r="Q18" s="10">
         <f t="shared" si="3"/>
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="R18" s="11"/>
     </row>
-    <row r="19" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
         <v>51</v>
       </c>
@@ -2997,7 +2991,7 @@
       <c r="M19" s="71">
         <v>1</v>
       </c>
-      <c r="N19" s="71">
+      <c r="N19" s="72">
         <v>1</v>
       </c>
       <c r="O19" s="10"/>
@@ -3011,7 +3005,7 @@
       </c>
       <c r="R19" s="11"/>
     </row>
-    <row r="20" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
         <v>51</v>
       </c>
@@ -3043,7 +3037,7 @@
       <c r="M20" s="71">
         <v>1</v>
       </c>
-      <c r="N20" s="71">
+      <c r="N20" s="72">
         <v>1</v>
       </c>
       <c r="O20" s="10"/>
@@ -3057,7 +3051,7 @@
       </c>
       <c r="R20" s="11"/>
     </row>
-    <row r="21" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
         <v>51</v>
       </c>
@@ -3089,7 +3083,7 @@
       <c r="M21" s="71">
         <v>1</v>
       </c>
-      <c r="N21" s="71">
+      <c r="N21" s="72">
         <v>1</v>
       </c>
       <c r="O21" s="10"/>
@@ -3103,7 +3097,7 @@
       </c>
       <c r="R21" s="11"/>
     </row>
-    <row r="22" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
         <v>51</v>
       </c>
@@ -3135,7 +3129,7 @@
       <c r="M22" s="71">
         <v>1</v>
       </c>
-      <c r="N22" s="71">
+      <c r="N22" s="72">
         <v>1</v>
       </c>
       <c r="O22" s="10"/>
@@ -3149,7 +3143,7 @@
       </c>
       <c r="R22" s="11"/>
     </row>
-    <row r="23" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
         <v>212</v>
       </c>
@@ -3194,12 +3188,12 @@
         <v>0.999</v>
       </c>
       <c r="Q23" s="60">
-        <f t="shared" ref="Q23:Q29" si="5">K23*N23</f>
+        <f t="shared" ref="Q23:Q30" si="5">K23*N23</f>
         <v>0.999</v>
       </c>
       <c r="R23" s="11"/>
     </row>
-    <row r="24" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
         <v>212</v>
       </c>
@@ -3249,7 +3243,7 @@
       </c>
       <c r="R24" s="11"/>
     </row>
-    <row r="25" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="12" t="s">
         <v>212</v>
       </c>
@@ -3299,7 +3293,7 @@
       </c>
       <c r="R25" s="11"/>
     </row>
-    <row r="26" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
         <v>212</v>
       </c>
@@ -3336,7 +3330,7 @@
       </c>
       <c r="R26" s="11"/>
     </row>
-    <row r="27" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
         <v>212</v>
       </c>
@@ -3384,7 +3378,7 @@
       </c>
       <c r="R27" s="11"/>
     </row>
-    <row r="28" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="12" t="s">
         <v>212</v>
       </c>
@@ -3434,7 +3428,7 @@
       </c>
       <c r="R28" s="11"/>
     </row>
-    <row r="29" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="12" t="s">
         <v>212</v>
       </c>
@@ -3484,7 +3478,7 @@
       </c>
       <c r="R29" s="11"/>
     </row>
-    <row r="30" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
         <v>212</v>
       </c>
@@ -3524,10 +3518,13 @@
         <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
-      <c r="Q30" s="11"/>
+      <c r="Q30" s="11">
+        <f t="shared" si="5"/>
+        <v>0.9</v>
+      </c>
       <c r="R30" s="28"/>
     </row>
-    <row r="31" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
         <v>212</v>
       </c>
@@ -3559,9 +3556,7 @@
       <c r="M31" s="17">
         <v>1</v>
       </c>
-      <c r="N31" s="17">
-        <v>1</v>
-      </c>
+      <c r="N31" s="17"/>
       <c r="O31" s="10"/>
       <c r="P31" s="10" t="e">
         <f t="shared" si="2"/>
@@ -3570,7 +3565,7 @@
       <c r="Q31" s="11"/>
       <c r="R31" s="11"/>
     </row>
-    <row r="32" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
         <v>212</v>
       </c>
@@ -3602,9 +3597,7 @@
       <c r="M32" s="17">
         <v>1</v>
       </c>
-      <c r="N32" s="17">
-        <v>1</v>
-      </c>
+      <c r="N32" s="17"/>
       <c r="O32" s="10"/>
       <c r="P32" s="10" t="e">
         <f t="shared" si="2"/>
@@ -3613,7 +3606,7 @@
       <c r="Q32" s="11"/>
       <c r="R32" s="11"/>
     </row>
-    <row r="33" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
         <v>212</v>
       </c>
@@ -3645,9 +3638,7 @@
       <c r="M33" s="17">
         <v>1</v>
       </c>
-      <c r="N33" s="17">
-        <v>1</v>
-      </c>
+      <c r="N33" s="17"/>
       <c r="O33" s="10"/>
       <c r="P33" s="10" t="e">
         <f t="shared" si="2"/>
@@ -3656,7 +3647,7 @@
       <c r="Q33" s="11"/>
       <c r="R33" s="11"/>
     </row>
-    <row r="34" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
         <v>212</v>
       </c>
@@ -3688,9 +3679,7 @@
       <c r="M34" s="17">
         <v>1</v>
       </c>
-      <c r="N34" s="17">
-        <v>1</v>
-      </c>
+      <c r="N34" s="17"/>
       <c r="O34" s="10"/>
       <c r="P34" s="10" t="e">
         <f t="shared" si="2"/>
@@ -3699,7 +3688,7 @@
       <c r="Q34" s="11"/>
       <c r="R34" s="11"/>
     </row>
-    <row r="35" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="12" t="s">
         <v>212</v>
       </c>
@@ -3731,9 +3720,7 @@
       <c r="M35" s="17">
         <v>1</v>
       </c>
-      <c r="N35" s="17">
-        <v>1</v>
-      </c>
+      <c r="N35" s="17"/>
       <c r="O35" s="10"/>
       <c r="P35" s="10">
         <f t="shared" si="2"/>
@@ -3742,7 +3729,7 @@
       <c r="Q35" s="11"/>
       <c r="R35" s="11"/>
     </row>
-    <row r="36" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:18" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
         <v>212</v>
       </c>
@@ -3778,9 +3765,7 @@
       <c r="M36" s="17">
         <v>1</v>
       </c>
-      <c r="N36" s="17">
-        <v>1</v>
-      </c>
+      <c r="N36" s="17"/>
       <c r="O36" s="10"/>
       <c r="P36" s="60">
         <f t="shared" si="2"/>
@@ -3788,11 +3773,11 @@
       </c>
       <c r="Q36" s="60">
         <f>K36*N36</f>
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="R36" s="29"/>
     </row>
-    <row r="37" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
         <v>309</v>
       </c>
@@ -3835,7 +3820,7 @@
       <c r="Q37" s="11"/>
       <c r="R37" s="11"/>
     </row>
-    <row r="38" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
         <v>309</v>
       </c>
@@ -3876,7 +3861,7 @@
       <c r="Q38" s="11"/>
       <c r="R38" s="11"/>
     </row>
-    <row r="39" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="12" t="s">
         <v>226</v>
       </c>
@@ -3921,7 +3906,7 @@
       <c r="Q39" s="11"/>
       <c r="R39" s="11"/>
     </row>
-    <row r="40" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="12" t="s">
         <v>226</v>
       </c>
@@ -3967,7 +3952,7 @@
       </c>
       <c r="R40" s="11"/>
     </row>
-    <row r="41" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="12" t="s">
         <v>226</v>
       </c>
@@ -4010,7 +3995,7 @@
       <c r="Q41" s="11"/>
       <c r="R41" s="11"/>
     </row>
-    <row r="42" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="12" t="s">
         <v>226</v>
       </c>
@@ -4053,7 +4038,7 @@
       <c r="Q42" s="11"/>
       <c r="R42" s="11"/>
     </row>
-    <row r="43" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="12" t="s">
         <v>212</v>
       </c>
@@ -4096,7 +4081,7 @@
       <c r="Q43" s="11"/>
       <c r="R43" s="11"/>
     </row>
-    <row r="44" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="12" t="s">
         <v>212</v>
       </c>
@@ -4139,7 +4124,7 @@
       <c r="Q44" s="11"/>
       <c r="R44" s="11"/>
     </row>
-    <row r="45" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
         <v>226</v>
       </c>
@@ -4176,7 +4161,7 @@
         <v>2</v>
       </c>
       <c r="N45" s="71">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="O45" s="10"/>
       <c r="P45" s="10">
@@ -4185,11 +4170,11 @@
       </c>
       <c r="Q45" s="10">
         <f>K45*N45</f>
-        <v>0.5</v>
+        <v>0.375</v>
       </c>
       <c r="R45" s="11"/>
     </row>
-    <row r="46" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
         <v>226</v>
       </c>
@@ -4239,7 +4224,7 @@
       </c>
       <c r="R46" s="11"/>
     </row>
-    <row r="47" spans="1:18" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18" s="4" customFormat="1" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
         <v>226</v>
       </c>
@@ -4282,7 +4267,7 @@
       <c r="Q47" s="11"/>
       <c r="R47" s="11"/>
     </row>
-    <row r="48" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
         <v>226</v>
       </c>
@@ -4321,7 +4306,7 @@
       <c r="Q48" s="11"/>
       <c r="R48" s="11"/>
     </row>
-    <row r="49" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="12" t="s">
         <v>226</v>
       </c>
@@ -4364,7 +4349,7 @@
       <c r="Q49" s="10"/>
       <c r="R49" s="11"/>
     </row>
-    <row r="50" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="12" t="s">
         <v>226</v>
       </c>
@@ -4411,7 +4396,7 @@
       <c r="Q50" s="11"/>
       <c r="R50" s="11"/>
     </row>
-    <row r="51" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
         <v>226</v>
       </c>
@@ -4456,7 +4441,7 @@
       <c r="Q51" s="11"/>
       <c r="R51" s="11"/>
     </row>
-    <row r="52" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="12" t="s">
         <v>226</v>
       </c>
@@ -4503,7 +4488,7 @@
       <c r="Q52" s="11"/>
       <c r="R52" s="11"/>
     </row>
-    <row r="53" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
         <v>226</v>
       </c>
@@ -4549,7 +4534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="12" t="s">
         <v>226</v>
       </c>
@@ -4592,7 +4577,7 @@
       <c r="Q54" s="11"/>
       <c r="R54" s="11"/>
     </row>
-    <row r="55" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="12" t="s">
         <v>226</v>
       </c>
@@ -4635,7 +4620,7 @@
       <c r="Q55" s="11"/>
       <c r="R55" s="11"/>
     </row>
-    <row r="56" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="12" t="s">
         <v>226</v>
       </c>
@@ -4675,7 +4660,7 @@
       <c r="Q56" s="11"/>
       <c r="R56" s="11"/>
     </row>
-    <row r="57" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="12" t="s">
         <v>51</v>
       </c>
@@ -4718,7 +4703,7 @@
       <c r="Q57" s="11"/>
       <c r="R57" s="11"/>
     </row>
-    <row r="58" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="12" t="s">
         <v>51</v>
       </c>
@@ -4845,9 +4830,7 @@
       <c r="M60" s="17">
         <v>1</v>
       </c>
-      <c r="N60" s="17">
-        <v>1</v>
-      </c>
+      <c r="N60" s="17"/>
       <c r="O60" s="10"/>
       <c r="P60" s="10"/>
       <c r="Q60" s="11"/>
@@ -4889,9 +4872,7 @@
       <c r="M61" s="17">
         <v>1</v>
       </c>
-      <c r="N61" s="17">
-        <v>1</v>
-      </c>
+      <c r="N61" s="17"/>
       <c r="O61" s="10"/>
       <c r="P61" s="10"/>
       <c r="Q61" s="11"/>
@@ -5020,9 +5001,7 @@
       <c r="M64" s="17">
         <v>1</v>
       </c>
-      <c r="N64" s="17">
-        <v>1</v>
-      </c>
+      <c r="N64" s="17"/>
       <c r="O64" s="10"/>
       <c r="P64" s="10">
         <f t="shared" ref="P64:P69" si="7">K64*M64</f>
@@ -5063,9 +5042,7 @@
       <c r="M65" s="17">
         <v>1</v>
       </c>
-      <c r="N65" s="17">
-        <v>1</v>
-      </c>
+      <c r="N65" s="17"/>
       <c r="O65" s="10"/>
       <c r="P65" s="10">
         <f t="shared" si="7"/>
@@ -5106,9 +5083,7 @@
       <c r="M66" s="17">
         <v>1</v>
       </c>
-      <c r="N66" s="17">
-        <v>1</v>
-      </c>
+      <c r="N66" s="17"/>
       <c r="O66" s="10"/>
       <c r="P66" s="10">
         <f t="shared" si="7"/>
@@ -5153,9 +5128,7 @@
       <c r="M67" s="17">
         <v>1</v>
       </c>
-      <c r="N67" s="17">
-        <v>1</v>
-      </c>
+      <c r="N67" s="17"/>
       <c r="O67" s="10"/>
       <c r="P67" s="10">
         <f t="shared" si="7"/>
@@ -5200,9 +5173,7 @@
       <c r="M68" s="17">
         <v>1</v>
       </c>
-      <c r="N68" s="17">
-        <v>1</v>
-      </c>
+      <c r="N68" s="17"/>
       <c r="O68" s="10"/>
       <c r="P68" s="10">
         <f t="shared" si="7"/>
@@ -5211,7 +5182,7 @@
       <c r="Q68" s="11"/>
       <c r="R68" s="11"/>
     </row>
-    <row r="69" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:18" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="43" t="s">
         <v>226</v>
       </c>
@@ -5246,7 +5217,7 @@
       <c r="Q69" s="11"/>
       <c r="R69" s="28"/>
     </row>
-    <row r="70" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:18" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="31"/>
       <c r="B70" s="31"/>
       <c r="C70" s="31"/>
@@ -5267,7 +5238,14 @@
       <c r="R70" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R70" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R70" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="WALI"/>
+        <filter val="WASO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="G24">
     <cfRule type="colorScale" priority="31">
       <colorScale>
@@ -5472,7 +5450,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M9:N10 M12:N22 M37:N42 M45:N45">
+  <conditionalFormatting sqref="M9:N10 M37:N42 M45:N45 M12:N22">
     <cfRule type="colorScale" priority="42">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
update baseline & other sectors ndc3.0
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_morocco_transformation_cw.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_morocco_transformation_cw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_morocco/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9016A1-B107-B04D-8BAE-80DC2376C6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C70528-5854-714D-9E94-0EFCF8C3B0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2114,7 +2114,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:R70"/>
@@ -2183,7 +2183,7 @@
       <c r="Q1" s="11"/>
       <c r="R1" s="11"/>
     </row>
-    <row r="2" spans="1:18" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" s="4" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>212</v>
       </c>
@@ -2222,7 +2222,7 @@
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
     </row>
-    <row r="3" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>212</v>
       </c>
@@ -2263,7 +2263,7 @@
       <c r="Q3" s="11"/>
       <c r="R3" s="11"/>
     </row>
-    <row r="4" spans="1:18" s="4" customFormat="1" ht="86" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" s="4" customFormat="1" ht="86" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>212</v>
       </c>
@@ -2304,7 +2304,7 @@
       </c>
       <c r="R4" s="11"/>
     </row>
-    <row r="5" spans="1:18" s="4" customFormat="1" ht="153" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" s="4" customFormat="1" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>212</v>
       </c>
@@ -2343,7 +2343,7 @@
       <c r="Q5" s="11"/>
       <c r="R5" s="11"/>
     </row>
-    <row r="6" spans="1:18" s="4" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" s="4" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>212</v>
       </c>
@@ -2389,7 +2389,7 @@
       </c>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
         <v>226</v>
       </c>
@@ -2430,7 +2430,7 @@
       <c r="Q7" s="11"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" s="4" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" s="4" customFormat="1" ht="55" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>226</v>
       </c>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>226</v>
       </c>
@@ -2527,7 +2527,7 @@
       <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
     </row>
-    <row r="10" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>226</v>
       </c>
@@ -2574,7 +2574,7 @@
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
     </row>
-    <row r="11" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
         <v>226</v>
       </c>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="R11" s="11"/>
     </row>
-    <row r="12" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>226</v>
       </c>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
         <v>226</v>
       </c>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="R13" s="11"/>
     </row>
-    <row r="14" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>226</v>
       </c>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="R14" s="11"/>
     </row>
-    <row r="15" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
         <v>226</v>
       </c>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="R15" s="11"/>
     </row>
-    <row r="16" spans="1:18" s="4" customFormat="1" ht="114" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" s="4" customFormat="1" ht="114" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
         <v>226</v>
       </c>
@@ -2835,7 +2835,7 @@
       <c r="Q16" s="11"/>
       <c r="R16" s="11"/>
     </row>
-    <row r="17" spans="1:18" s="58" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" s="58" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="s">
         <v>51</v>
       </c>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="R17" s="57"/>
     </row>
-    <row r="18" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
         <v>51</v>
       </c>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="R18" s="11"/>
     </row>
-    <row r="19" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
         <v>51</v>
       </c>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="R19" s="11"/>
     </row>
-    <row r="20" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
         <v>51</v>
       </c>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="R20" s="11"/>
     </row>
-    <row r="21" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
         <v>51</v>
       </c>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="R21" s="11"/>
     </row>
-    <row r="22" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
         <v>51</v>
       </c>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="R22" s="11"/>
     </row>
-    <row r="23" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
         <v>212</v>
       </c>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="R23" s="11"/>
     </row>
-    <row r="24" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
         <v>212</v>
       </c>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="R24" s="11"/>
     </row>
-    <row r="25" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="12" t="s">
         <v>212</v>
       </c>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="R25" s="11"/>
     </row>
-    <row r="26" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
         <v>212</v>
       </c>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="R26" s="11"/>
     </row>
-    <row r="27" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
         <v>212</v>
       </c>
@@ -3340,7 +3340,7 @@
       </c>
       <c r="R27" s="11"/>
     </row>
-    <row r="28" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="12" t="s">
         <v>212</v>
       </c>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="R28" s="11"/>
     </row>
-    <row r="29" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="12" t="s">
         <v>212</v>
       </c>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="R29" s="11"/>
     </row>
-    <row r="30" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
         <v>212</v>
       </c>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="R30" s="28"/>
     </row>
-    <row r="31" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
         <v>212</v>
       </c>
@@ -3519,7 +3519,7 @@
       <c r="Q31" s="11"/>
       <c r="R31" s="11"/>
     </row>
-    <row r="32" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
         <v>212</v>
       </c>
@@ -3558,7 +3558,7 @@
       <c r="Q32" s="11"/>
       <c r="R32" s="11"/>
     </row>
-    <row r="33" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
         <v>212</v>
       </c>
@@ -3597,7 +3597,7 @@
       <c r="Q33" s="11"/>
       <c r="R33" s="11"/>
     </row>
-    <row r="34" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
         <v>212</v>
       </c>
@@ -3636,7 +3636,7 @@
       <c r="Q34" s="11"/>
       <c r="R34" s="11"/>
     </row>
-    <row r="35" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="12" t="s">
         <v>212</v>
       </c>
@@ -3675,7 +3675,7 @@
       <c r="Q35" s="11"/>
       <c r="R35" s="11"/>
     </row>
-    <row r="36" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:18" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
         <v>212</v>
       </c>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="R36" s="29"/>
     </row>
-    <row r="37" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
         <v>309</v>
       </c>
@@ -3762,7 +3762,7 @@
       <c r="Q37" s="11"/>
       <c r="R37" s="11"/>
     </row>
-    <row r="38" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
         <v>309</v>
       </c>
@@ -3803,7 +3803,7 @@
       <c r="Q38" s="11"/>
       <c r="R38" s="11"/>
     </row>
-    <row r="39" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="12" t="s">
         <v>226</v>
       </c>
@@ -3846,7 +3846,7 @@
       <c r="Q39" s="11"/>
       <c r="R39" s="11"/>
     </row>
-    <row r="40" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="12" t="s">
         <v>226</v>
       </c>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="R40" s="11"/>
     </row>
-    <row r="41" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="12" t="s">
         <v>226</v>
       </c>
@@ -3931,7 +3931,7 @@
       <c r="Q41" s="11"/>
       <c r="R41" s="11"/>
     </row>
-    <row r="42" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="12" t="s">
         <v>226</v>
       </c>
@@ -3962,17 +3962,20 @@
       </c>
       <c r="M42" s="71"/>
       <c r="N42" s="71">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="O42" s="10"/>
       <c r="P42" s="10">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Q42" s="11"/>
+      <c r="Q42" s="10">
+        <f>K42*N42</f>
+        <v>0.90249999999999997</v>
+      </c>
       <c r="R42" s="11"/>
     </row>
-    <row r="43" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="12" t="s">
         <v>212</v>
       </c>
@@ -4013,7 +4016,7 @@
       <c r="Q43" s="11"/>
       <c r="R43" s="11"/>
     </row>
-    <row r="44" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="12" t="s">
         <v>212</v>
       </c>
@@ -4057,7 +4060,7 @@
       </c>
       <c r="R44" s="11"/>
     </row>
-    <row r="45" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
         <v>226</v>
       </c>
@@ -4105,7 +4108,7 @@
       </c>
       <c r="R45" s="11"/>
     </row>
-    <row r="46" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
         <v>226</v>
       </c>
@@ -4153,7 +4156,7 @@
       </c>
       <c r="R46" s="11"/>
     </row>
-    <row r="47" spans="1:18" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18" s="4" customFormat="1" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
         <v>226</v>
       </c>
@@ -4196,7 +4199,7 @@
       <c r="Q47" s="11"/>
       <c r="R47" s="11"/>
     </row>
-    <row r="48" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
         <v>226</v>
       </c>
@@ -4235,7 +4238,7 @@
       <c r="Q48" s="11"/>
       <c r="R48" s="11"/>
     </row>
-    <row r="49" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="12" t="s">
         <v>226</v>
       </c>
@@ -4276,7 +4279,7 @@
       <c r="Q49" s="10"/>
       <c r="R49" s="11"/>
     </row>
-    <row r="50" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="12" t="s">
         <v>226</v>
       </c>
@@ -4321,7 +4324,7 @@
       <c r="Q50" s="11"/>
       <c r="R50" s="11"/>
     </row>
-    <row r="51" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
         <v>226</v>
       </c>
@@ -4364,7 +4367,7 @@
       <c r="Q51" s="11"/>
       <c r="R51" s="11"/>
     </row>
-    <row r="52" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="12" t="s">
         <v>226</v>
       </c>
@@ -4409,7 +4412,7 @@
       <c r="Q52" s="11"/>
       <c r="R52" s="11"/>
     </row>
-    <row r="53" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
         <v>226</v>
       </c>
@@ -4453,7 +4456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="12" t="s">
         <v>226</v>
       </c>
@@ -4496,7 +4499,7 @@
       <c r="Q54" s="11"/>
       <c r="R54" s="11"/>
     </row>
-    <row r="55" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="12" t="s">
         <v>226</v>
       </c>
@@ -4539,7 +4542,7 @@
       <c r="Q55" s="11"/>
       <c r="R55" s="11"/>
     </row>
-    <row r="56" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="12" t="s">
         <v>226</v>
       </c>
@@ -5077,7 +5080,7 @@
       <c r="Q68" s="11"/>
       <c r="R68" s="11"/>
     </row>
-    <row r="69" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:18" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="43" t="s">
         <v>226</v>
       </c>
@@ -5112,7 +5115,7 @@
       <c r="Q69" s="11"/>
       <c r="R69" s="28"/>
     </row>
-    <row r="70" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:18" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="31"/>
       <c r="B70" s="31"/>
       <c r="C70" s="31"/>
@@ -5133,7 +5136,15 @@
       <c r="R70" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R70" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R70" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="TRWW"/>
+        <filter val="WALI"/>
+        <filter val="WASO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="G24">
     <cfRule type="colorScale" priority="32">
       <colorScale>

</xml_diff>